<commit_message>
Update GUS trade data for 2019
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2018_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2019_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2018_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2019_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -586,6 +586,19 @@
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -679,6 +692,71 @@
           <t>2018 M12</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M01</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M02</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M03</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M04</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M05</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M06</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M07</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M08</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M09</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M10</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M11</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -744,6 +822,45 @@
       </c>
       <c r="R2" s="3" t="n">
         <v>75759807328</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>1018478990123</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>81878946831</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>84262405536</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>87102444456</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>84976653564</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>88383931681</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>79441568926</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>85302840577</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>79596187291</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>86733941116</v>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>95273020159</v>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v>87916978261</v>
+      </c>
+      <c r="AE2" s="3" t="n">
+        <v>77610071725</v>
       </c>
     </row>
   </sheetData>
@@ -757,7 +874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -778,6 +895,19 @@
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="11" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -871,6 +1001,71 @@
           <t>2018 M12</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M01</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M02</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M03</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M04</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M05</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M06</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M07</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M08</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M09</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M10</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M11</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -936,6 +1131,45 @@
       </c>
       <c r="R2" s="3" t="n">
         <v>-5980263360</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>5112453119</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>733726052</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>-1954825180</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>2496930291</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>585921776</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>-1061826295</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>411785338</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>-529644948</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>-1092973002</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>2702466384</v>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>978564891</v>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v>2307194932</v>
+      </c>
+      <c r="AE2" s="3" t="n">
+        <v>-464867120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GUS trade data for 2020
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2019_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2020_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2019_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2020_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -599,6 +599,19 @@
     <col width="13" customWidth="1" min="29" max="29"/>
     <col width="13" customWidth="1" min="30" max="30"/>
     <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="15" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="13" customWidth="1" min="42" max="42"/>
+    <col width="13" customWidth="1" min="43" max="43"/>
+    <col width="13" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -757,6 +770,71 @@
           <t>2019 M12</t>
         </is>
       </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M01</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M02</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M03</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M04</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M05</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M06</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M07</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M08</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M09</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M10</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M11</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -861,6 +939,45 @@
       </c>
       <c r="AE2" s="3" t="n">
         <v>77610071725</v>
+      </c>
+      <c r="AF2" s="3" t="n">
+        <v>1015359469371</v>
+      </c>
+      <c r="AG2" s="3" t="n">
+        <v>85719340057</v>
+      </c>
+      <c r="AH2" s="3" t="n">
+        <v>85322004582</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>88630065031</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>65723949702</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>68818787951</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>76534316206</v>
+      </c>
+      <c r="AM2" s="3" t="n">
+        <v>86807041070</v>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v>77880800695</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>92423974871</v>
+      </c>
+      <c r="AP2" s="3" t="n">
+        <v>99148459206</v>
+      </c>
+      <c r="AQ2" s="3" t="n">
+        <v>98581138974</v>
+      </c>
+      <c r="AR2" s="3" t="n">
+        <v>89769591026</v>
       </c>
     </row>
   </sheetData>
@@ -874,7 +991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -908,6 +1025,19 @@
     <col width="11" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="39" max="39"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1066,6 +1196,71 @@
           <t>2019 M12</t>
         </is>
       </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M01</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M02</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M03</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M04</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M05</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M06</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M07</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M08</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M09</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M10</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M11</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1170,6 +1365,45 @@
       </c>
       <c r="AE2" s="3" t="n">
         <v>-464867120</v>
+      </c>
+      <c r="AF2" s="3" t="n">
+        <v>47154049085</v>
+      </c>
+      <c r="AG2" s="3" t="n">
+        <v>388407522</v>
+      </c>
+      <c r="AH2" s="3" t="n">
+        <v>2709752292</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>-620703289</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>-1184794007</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>4954730141</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>10448837246</v>
+      </c>
+      <c r="AM2" s="3" t="n">
+        <v>2500047349</v>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v>3958561838</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>6715743455</v>
+      </c>
+      <c r="AP2" s="3" t="n">
+        <v>7804181198</v>
+      </c>
+      <c r="AQ2" s="3" t="n">
+        <v>7540400965</v>
+      </c>
+      <c r="AR2" s="3" t="n">
+        <v>1938884375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GUS trade data for 2021
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2020_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2021_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2020_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2021_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR2"/>
+  <dimension ref="A1:BE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -612,6 +612,19 @@
     <col width="13" customWidth="1" min="42" max="42"/>
     <col width="13" customWidth="1" min="43" max="43"/>
     <col width="13" customWidth="1" min="44" max="44"/>
+    <col width="15" customWidth="1" min="45" max="45"/>
+    <col width="13" customWidth="1" min="46" max="46"/>
+    <col width="13" customWidth="1" min="47" max="47"/>
+    <col width="14" customWidth="1" min="48" max="48"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="14" customWidth="1" min="50" max="50"/>
+    <col width="14" customWidth="1" min="51" max="51"/>
+    <col width="14" customWidth="1" min="52" max="52"/>
+    <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -835,6 +848,71 @@
           <t>2020 M12</t>
         </is>
       </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M01</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M02</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M03</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M04</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M05</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M06</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M07</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M08</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M09</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M10</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M11</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -978,6 +1056,45 @@
       </c>
       <c r="AR2" s="3" t="n">
         <v>89769591026</v>
+      </c>
+      <c r="AS2" s="3" t="n">
+        <v>1322836427065</v>
+      </c>
+      <c r="AT2" s="3" t="n">
+        <v>87308509835</v>
+      </c>
+      <c r="AU2" s="3" t="n">
+        <v>96304162617</v>
+      </c>
+      <c r="AV2" s="3" t="n">
+        <v>113215898683</v>
+      </c>
+      <c r="AW2" s="3" t="n">
+        <v>102413806676</v>
+      </c>
+      <c r="AX2" s="3" t="n">
+        <v>105007555982</v>
+      </c>
+      <c r="AY2" s="3" t="n">
+        <v>107522422207</v>
+      </c>
+      <c r="AZ2" s="3" t="n">
+        <v>109176414628</v>
+      </c>
+      <c r="BA2" s="3" t="n">
+        <v>107114339770</v>
+      </c>
+      <c r="BB2" s="3" t="n">
+        <v>115206510396</v>
+      </c>
+      <c r="BC2" s="3" t="n">
+        <v>120781698204</v>
+      </c>
+      <c r="BD2" s="3" t="n">
+        <v>131750859209</v>
+      </c>
+      <c r="BE2" s="3" t="n">
+        <v>127034248858</v>
       </c>
     </row>
   </sheetData>
@@ -991,7 +1108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR2"/>
+  <dimension ref="A1:BE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1038,6 +1155,19 @@
     <col width="12" customWidth="1" min="42" max="42"/>
     <col width="12" customWidth="1" min="43" max="43"/>
     <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="13" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
+    <col width="12" customWidth="1" min="47" max="47"/>
+    <col width="12" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
+    <col width="12" customWidth="1" min="50" max="50"/>
+    <col width="12" customWidth="1" min="51" max="51"/>
+    <col width="13" customWidth="1" min="52" max="52"/>
+    <col width="13" customWidth="1" min="53" max="53"/>
+    <col width="13" customWidth="1" min="54" max="54"/>
+    <col width="13" customWidth="1" min="55" max="55"/>
+    <col width="13" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1261,6 +1391,71 @@
           <t>2020 M12</t>
         </is>
       </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M01</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M02</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M03</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M04</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M05</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M06</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M07</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M08</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M09</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M10</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M11</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1404,6 +1599,45 @@
       </c>
       <c r="AR2" s="3" t="n">
         <v>1938884375</v>
+      </c>
+      <c r="AS2" s="3" t="n">
+        <v>-6858605920</v>
+      </c>
+      <c r="AT2" s="3" t="n">
+        <v>5589699811</v>
+      </c>
+      <c r="AU2" s="3" t="n">
+        <v>2421564871</v>
+      </c>
+      <c r="AV2" s="3" t="n">
+        <v>2254839081</v>
+      </c>
+      <c r="AW2" s="3" t="n">
+        <v>6689022728</v>
+      </c>
+      <c r="AX2" s="3" t="n">
+        <v>-269004710</v>
+      </c>
+      <c r="AY2" s="3" t="n">
+        <v>1902719382</v>
+      </c>
+      <c r="AZ2" s="3" t="n">
+        <v>-2854752437</v>
+      </c>
+      <c r="BA2" s="3" t="n">
+        <v>-5412113866</v>
+      </c>
+      <c r="BB2" s="3" t="n">
+        <v>-1138520594</v>
+      </c>
+      <c r="BC2" s="3" t="n">
+        <v>-1483951182</v>
+      </c>
+      <c r="BD2" s="3" t="n">
+        <v>-1997978923</v>
+      </c>
+      <c r="BE2" s="3" t="n">
+        <v>-12560130081</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GUS trade data for 2022
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2021_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2022_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2021_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2022_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE2"/>
+  <dimension ref="A1:BR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -625,6 +625,19 @@
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="14" customWidth="1" min="56" max="56"/>
     <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="15" customWidth="1" min="58" max="58"/>
+    <col width="14" customWidth="1" min="59" max="59"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
+    <col width="14" customWidth="1" min="61" max="61"/>
+    <col width="14" customWidth="1" min="62" max="62"/>
+    <col width="14" customWidth="1" min="63" max="63"/>
+    <col width="14" customWidth="1" min="64" max="64"/>
+    <col width="14" customWidth="1" min="65" max="65"/>
+    <col width="14" customWidth="1" min="66" max="66"/>
+    <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="14" customWidth="1" min="68" max="68"/>
+    <col width="14" customWidth="1" min="69" max="69"/>
+    <col width="14" customWidth="1" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -913,6 +926,71 @@
           <t>2021 M12</t>
         </is>
       </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M01</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M02</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M03</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M04</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M05</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M06</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M07</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M08</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M09</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M10</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M11</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1095,6 +1173,45 @@
       </c>
       <c r="BE2" s="3" t="n">
         <v>127034248858</v>
+      </c>
+      <c r="BF2" s="3" t="n">
+        <v>1711761281378</v>
+      </c>
+      <c r="BG2" s="3" t="n">
+        <v>118102079385</v>
+      </c>
+      <c r="BH2" s="3" t="n">
+        <v>124248800187</v>
+      </c>
+      <c r="BI2" s="3" t="n">
+        <v>151726073482</v>
+      </c>
+      <c r="BJ2" s="3" t="n">
+        <v>139989330211</v>
+      </c>
+      <c r="BK2" s="3" t="n">
+        <v>141548686152</v>
+      </c>
+      <c r="BL2" s="3" t="n">
+        <v>140830232343</v>
+      </c>
+      <c r="BM2" s="3" t="n">
+        <v>138460636738</v>
+      </c>
+      <c r="BN2" s="3" t="n">
+        <v>142353469663</v>
+      </c>
+      <c r="BO2" s="3" t="n">
+        <v>156928695934</v>
+      </c>
+      <c r="BP2" s="3" t="n">
+        <v>158781327131</v>
+      </c>
+      <c r="BQ2" s="3" t="n">
+        <v>156923020047</v>
+      </c>
+      <c r="BR2" s="3" t="n">
+        <v>141868930105</v>
       </c>
     </row>
   </sheetData>
@@ -1108,7 +1225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE2"/>
+  <dimension ref="A1:BR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1168,6 +1285,19 @@
     <col width="13" customWidth="1" min="55" max="55"/>
     <col width="13" customWidth="1" min="56" max="56"/>
     <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
+    <col width="12" customWidth="1" min="59" max="59"/>
+    <col width="13" customWidth="1" min="60" max="60"/>
+    <col width="14" customWidth="1" min="61" max="61"/>
+    <col width="14" customWidth="1" min="62" max="62"/>
+    <col width="13" customWidth="1" min="63" max="63"/>
+    <col width="13" customWidth="1" min="64" max="64"/>
+    <col width="13" customWidth="1" min="65" max="65"/>
+    <col width="14" customWidth="1" min="66" max="66"/>
+    <col width="14" customWidth="1" min="67" max="67"/>
+    <col width="13" customWidth="1" min="68" max="68"/>
+    <col width="12" customWidth="1" min="69" max="69"/>
+    <col width="14" customWidth="1" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1456,6 +1586,71 @@
           <t>2021 M12</t>
         </is>
       </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M01</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M02</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M03</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M04</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M05</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M06</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M07</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M08</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M09</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M10</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M11</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1638,6 +1833,45 @@
       </c>
       <c r="BE2" s="3" t="n">
         <v>-12560130081</v>
+      </c>
+      <c r="BF2" s="3" t="n">
+        <v>-93202074819</v>
+      </c>
+      <c r="BG2" s="3" t="n">
+        <v>-765996889</v>
+      </c>
+      <c r="BH2" s="3" t="n">
+        <v>-4661828520</v>
+      </c>
+      <c r="BI2" s="3" t="n">
+        <v>-16218109261</v>
+      </c>
+      <c r="BJ2" s="3" t="n">
+        <v>-11562431704</v>
+      </c>
+      <c r="BK2" s="3" t="n">
+        <v>-5055901167</v>
+      </c>
+      <c r="BL2" s="3" t="n">
+        <v>-4165894473</v>
+      </c>
+      <c r="BM2" s="3" t="n">
+        <v>-7414574345</v>
+      </c>
+      <c r="BN2" s="3" t="n">
+        <v>-10243100752</v>
+      </c>
+      <c r="BO2" s="3" t="n">
+        <v>-10389008143</v>
+      </c>
+      <c r="BP2" s="3" t="n">
+        <v>-8322085235</v>
+      </c>
+      <c r="BQ2" s="3" t="n">
+        <v>-823289922</v>
+      </c>
+      <c r="BR2" s="3" t="n">
+        <v>-13579854408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GUS trade data for 2023
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2022_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2023_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2022_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2023_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR2"/>
+  <dimension ref="A1:CE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -638,6 +638,19 @@
     <col width="14" customWidth="1" min="68" max="68"/>
     <col width="14" customWidth="1" min="69" max="69"/>
     <col width="14" customWidth="1" min="70" max="70"/>
+    <col width="15" customWidth="1" min="71" max="71"/>
+    <col width="14" customWidth="1" min="72" max="72"/>
+    <col width="14" customWidth="1" min="73" max="73"/>
+    <col width="14" customWidth="1" min="74" max="74"/>
+    <col width="14" customWidth="1" min="75" max="75"/>
+    <col width="14" customWidth="1" min="76" max="76"/>
+    <col width="14" customWidth="1" min="77" max="77"/>
+    <col width="14" customWidth="1" min="78" max="78"/>
+    <col width="14" customWidth="1" min="79" max="79"/>
+    <col width="14" customWidth="1" min="80" max="80"/>
+    <col width="14" customWidth="1" min="81" max="81"/>
+    <col width="14" customWidth="1" min="82" max="82"/>
+    <col width="14" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -991,6 +1004,71 @@
           <t>2022 M12</t>
         </is>
       </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M01</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M02</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M03</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M04</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M05</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M06</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M07</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M08</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M09</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M10</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M11</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1212,6 +1290,45 @@
       </c>
       <c r="BR2" s="3" t="n">
         <v>141868930105</v>
+      </c>
+      <c r="BS2" s="3" t="n">
+        <v>1568329175183</v>
+      </c>
+      <c r="BT2" s="3" t="n">
+        <v>135808799687</v>
+      </c>
+      <c r="BU2" s="3" t="n">
+        <v>132287310174</v>
+      </c>
+      <c r="BV2" s="3" t="n">
+        <v>148360593649</v>
+      </c>
+      <c r="BW2" s="3" t="n">
+        <v>128752171605</v>
+      </c>
+      <c r="BX2" s="3" t="n">
+        <v>131960375419</v>
+      </c>
+      <c r="BY2" s="3" t="n">
+        <v>128195849910</v>
+      </c>
+      <c r="BZ2" s="3" t="n">
+        <v>121573406362</v>
+      </c>
+      <c r="CA2" s="3" t="n">
+        <v>120031626529</v>
+      </c>
+      <c r="CB2" s="3" t="n">
+        <v>129667203351</v>
+      </c>
+      <c r="CC2" s="3" t="n">
+        <v>139369120258</v>
+      </c>
+      <c r="CD2" s="3" t="n">
+        <v>137198489260</v>
+      </c>
+      <c r="CE2" s="3" t="n">
+        <v>115124228979</v>
       </c>
     </row>
   </sheetData>
@@ -1225,7 +1342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR2"/>
+  <dimension ref="A1:CE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1298,6 +1415,19 @@
     <col width="13" customWidth="1" min="68" max="68"/>
     <col width="12" customWidth="1" min="69" max="69"/>
     <col width="14" customWidth="1" min="70" max="70"/>
+    <col width="13" customWidth="1" min="71" max="71"/>
+    <col width="12" customWidth="1" min="72" max="72"/>
+    <col width="12" customWidth="1" min="73" max="73"/>
+    <col width="12" customWidth="1" min="74" max="74"/>
+    <col width="12" customWidth="1" min="75" max="75"/>
+    <col width="12" customWidth="1" min="76" max="76"/>
+    <col width="12" customWidth="1" min="77" max="77"/>
+    <col width="12" customWidth="1" min="78" max="78"/>
+    <col width="12" customWidth="1" min="79" max="79"/>
+    <col width="12" customWidth="1" min="80" max="80"/>
+    <col width="12" customWidth="1" min="81" max="81"/>
+    <col width="12" customWidth="1" min="82" max="82"/>
+    <col width="13" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1651,6 +1781,71 @@
           <t>2022 M12</t>
         </is>
       </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M01</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M02</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M03</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M04</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M05</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M06</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M07</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M08</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M09</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M10</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M11</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1872,6 +2067,45 @@
       </c>
       <c r="BR2" s="3" t="n">
         <v>-13579854408</v>
+      </c>
+      <c r="BS2" s="3" t="n">
+        <v>45063921119</v>
+      </c>
+      <c r="BT2" s="3" t="n">
+        <v>3498138832</v>
+      </c>
+      <c r="BU2" s="3" t="n">
+        <v>4967591607</v>
+      </c>
+      <c r="BV2" s="3" t="n">
+        <v>7034358395</v>
+      </c>
+      <c r="BW2" s="3" t="n">
+        <v>2633409359</v>
+      </c>
+      <c r="BX2" s="3" t="n">
+        <v>5643072034</v>
+      </c>
+      <c r="BY2" s="3" t="n">
+        <v>7936888679</v>
+      </c>
+      <c r="BZ2" s="3" t="n">
+        <v>1574389394</v>
+      </c>
+      <c r="CA2" s="3" t="n">
+        <v>1271793893</v>
+      </c>
+      <c r="CB2" s="3" t="n">
+        <v>5087409074</v>
+      </c>
+      <c r="CC2" s="3" t="n">
+        <v>5814332677</v>
+      </c>
+      <c r="CD2" s="3" t="n">
+        <v>1882491518</v>
+      </c>
+      <c r="CE2" s="3" t="n">
+        <v>-2279954343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GUS trade data for 2024
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2023_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2024_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2023_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2024_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE2"/>
+  <dimension ref="A1:CR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -651,6 +651,19 @@
     <col width="14" customWidth="1" min="81" max="81"/>
     <col width="14" customWidth="1" min="82" max="82"/>
     <col width="14" customWidth="1" min="83" max="83"/>
+    <col width="15" customWidth="1" min="84" max="84"/>
+    <col width="14" customWidth="1" min="85" max="85"/>
+    <col width="14" customWidth="1" min="86" max="86"/>
+    <col width="14" customWidth="1" min="87" max="87"/>
+    <col width="14" customWidth="1" min="88" max="88"/>
+    <col width="14" customWidth="1" min="89" max="89"/>
+    <col width="14" customWidth="1" min="90" max="90"/>
+    <col width="14" customWidth="1" min="91" max="91"/>
+    <col width="14" customWidth="1" min="92" max="92"/>
+    <col width="14" customWidth="1" min="93" max="93"/>
+    <col width="14" customWidth="1" min="94" max="94"/>
+    <col width="14" customWidth="1" min="95" max="95"/>
+    <col width="14" customWidth="1" min="96" max="96"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1069,6 +1082,71 @@
           <t>2023 M12</t>
         </is>
       </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M01</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M02</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M03</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M04</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M05</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M06</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M07</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M08</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M09</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M10</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M11</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1329,6 +1407,45 @@
       </c>
       <c r="CE2" s="3" t="n">
         <v>115124228979</v>
+      </c>
+      <c r="CF2" s="3" t="n">
+        <v>1521021537878</v>
+      </c>
+      <c r="CG2" s="3" t="n">
+        <v>119674100771</v>
+      </c>
+      <c r="CH2" s="3" t="n">
+        <v>124356203018</v>
+      </c>
+      <c r="CI2" s="3" t="n">
+        <v>125944035020</v>
+      </c>
+      <c r="CJ2" s="3" t="n">
+        <v>128273694854</v>
+      </c>
+      <c r="CK2" s="3" t="n">
+        <v>122400909701</v>
+      </c>
+      <c r="CL2" s="3" t="n">
+        <v>125390063140</v>
+      </c>
+      <c r="CM2" s="3" t="n">
+        <v>128343920499</v>
+      </c>
+      <c r="CN2" s="3" t="n">
+        <v>121566524262</v>
+      </c>
+      <c r="CO2" s="3" t="n">
+        <v>128568087014</v>
+      </c>
+      <c r="CP2" s="3" t="n">
+        <v>141129170798</v>
+      </c>
+      <c r="CQ2" s="3" t="n">
+        <v>135933806724</v>
+      </c>
+      <c r="CR2" s="3" t="n">
+        <v>119441022077</v>
       </c>
     </row>
   </sheetData>
@@ -1342,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE2"/>
+  <dimension ref="A1:CR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1428,6 +1545,19 @@
     <col width="12" customWidth="1" min="81" max="81"/>
     <col width="12" customWidth="1" min="82" max="82"/>
     <col width="13" customWidth="1" min="83" max="83"/>
+    <col width="12" customWidth="1" min="84" max="84"/>
+    <col width="12" customWidth="1" min="85" max="85"/>
+    <col width="12" customWidth="1" min="86" max="86"/>
+    <col width="12" customWidth="1" min="87" max="87"/>
+    <col width="12" customWidth="1" min="88" max="88"/>
+    <col width="11" customWidth="1" min="89" max="89"/>
+    <col width="12" customWidth="1" min="90" max="90"/>
+    <col width="13" customWidth="1" min="91" max="91"/>
+    <col width="13" customWidth="1" min="92" max="92"/>
+    <col width="11" customWidth="1" min="93" max="93"/>
+    <col width="11" customWidth="1" min="94" max="94"/>
+    <col width="13" customWidth="1" min="95" max="95"/>
+    <col width="13" customWidth="1" min="96" max="96"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1846,6 +1976,71 @@
           <t>2023 M12</t>
         </is>
       </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M01</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M02</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M03</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M04</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M05</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M06</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M07</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M08</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M09</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M10</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M11</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2106,6 +2301,45 @@
       </c>
       <c r="CE2" s="3" t="n">
         <v>-2279954343</v>
+      </c>
+      <c r="CF2" s="3" t="n">
+        <v>2332285853</v>
+      </c>
+      <c r="CG2" s="3" t="n">
+        <v>6511433863</v>
+      </c>
+      <c r="CH2" s="3" t="n">
+        <v>3263804131</v>
+      </c>
+      <c r="CI2" s="3" t="n">
+        <v>4588289765</v>
+      </c>
+      <c r="CJ2" s="3" t="n">
+        <v>2347137246</v>
+      </c>
+      <c r="CK2" s="3" t="n">
+        <v>820211099</v>
+      </c>
+      <c r="CL2" s="3" t="n">
+        <v>-113247867</v>
+      </c>
+      <c r="CM2" s="3" t="n">
+        <v>-2384387909</v>
+      </c>
+      <c r="CN2" s="3" t="n">
+        <v>-6588643341</v>
+      </c>
+      <c r="CO2" s="3" t="n">
+        <v>819063386</v>
+      </c>
+      <c r="CP2" s="3" t="n">
+        <v>679952238</v>
+      </c>
+      <c r="CQ2" s="3" t="n">
+        <v>-1586140224</v>
+      </c>
+      <c r="CR2" s="3" t="n">
+        <v>-6025186534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GUS trade data for 2025
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
+++ b/gus_dbw_trade/gus_import_saldo_PLN_2018_plus_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>13</v>
@@ -521,7 +521,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/import_wysylka_PLN_2024_raw.csv</t>
+          <t>gus_dbw_trade/import_wysylka_PLN_2025_raw.csv</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -550,7 +550,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2024_raw.csv</t>
+          <t>gus_dbw_trade/saldo_pochodzenie_PLN_2025_raw.csv</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR2"/>
+  <dimension ref="A1:DE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -664,6 +664,19 @@
     <col width="14" customWidth="1" min="94" max="94"/>
     <col width="14" customWidth="1" min="95" max="95"/>
     <col width="14" customWidth="1" min="96" max="96"/>
+    <col width="15" customWidth="1" min="97" max="97"/>
+    <col width="14" customWidth="1" min="98" max="98"/>
+    <col width="14" customWidth="1" min="99" max="99"/>
+    <col width="14" customWidth="1" min="100" max="100"/>
+    <col width="14" customWidth="1" min="101" max="101"/>
+    <col width="14" customWidth="1" min="102" max="102"/>
+    <col width="14" customWidth="1" min="103" max="103"/>
+    <col width="14" customWidth="1" min="104" max="104"/>
+    <col width="14" customWidth="1" min="105" max="105"/>
+    <col width="14" customWidth="1" min="106" max="106"/>
+    <col width="14" customWidth="1" min="107" max="107"/>
+    <col width="14" customWidth="1" min="108" max="108"/>
+    <col width="14" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1147,6 +1160,71 @@
           <t>2024 M12</t>
         </is>
       </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M01</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M02</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M03</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M04</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M05</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M06</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M07</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M08</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M09</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M10</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M11</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1446,6 +1524,45 @@
       </c>
       <c r="CR2" s="3" t="n">
         <v>119441022077</v>
+      </c>
+      <c r="CS2" s="3" t="n">
+        <v>1579712186610</v>
+      </c>
+      <c r="CT2" s="3" t="n">
+        <v>129924572110</v>
+      </c>
+      <c r="CU2" s="3" t="n">
+        <v>124597961041</v>
+      </c>
+      <c r="CV2" s="3" t="n">
+        <v>136985007407</v>
+      </c>
+      <c r="CW2" s="3" t="n">
+        <v>133238916210</v>
+      </c>
+      <c r="CX2" s="3" t="n">
+        <v>132935118944</v>
+      </c>
+      <c r="CY2" s="3" t="n">
+        <v>128274905127</v>
+      </c>
+      <c r="CZ2" s="3" t="n">
+        <v>131319787391</v>
+      </c>
+      <c r="DA2" s="3" t="n">
+        <v>120638948167</v>
+      </c>
+      <c r="DB2" s="3" t="n">
+        <v>137760301212</v>
+      </c>
+      <c r="DC2" s="3" t="n">
+        <v>143456653365</v>
+      </c>
+      <c r="DD2" s="3" t="n">
+        <v>133555018842</v>
+      </c>
+      <c r="DE2" s="3" t="n">
+        <v>127024996794</v>
       </c>
     </row>
   </sheetData>
@@ -1459,7 +1576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR2"/>
+  <dimension ref="A1:DE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1558,6 +1675,19 @@
     <col width="11" customWidth="1" min="94" max="94"/>
     <col width="13" customWidth="1" min="95" max="95"/>
     <col width="13" customWidth="1" min="96" max="96"/>
+    <col width="14" customWidth="1" min="97" max="97"/>
+    <col width="13" customWidth="1" min="98" max="98"/>
+    <col width="12" customWidth="1" min="99" max="99"/>
+    <col width="13" customWidth="1" min="100" max="100"/>
+    <col width="13" customWidth="1" min="101" max="101"/>
+    <col width="13" customWidth="1" min="102" max="102"/>
+    <col width="12" customWidth="1" min="103" max="103"/>
+    <col width="13" customWidth="1" min="104" max="104"/>
+    <col width="13" customWidth="1" min="105" max="105"/>
+    <col width="12" customWidth="1" min="106" max="106"/>
+    <col width="12" customWidth="1" min="107" max="107"/>
+    <col width="12" customWidth="1" min="108" max="108"/>
+    <col width="13" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2041,6 +2171,71 @@
           <t>2024 M12</t>
         </is>
       </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M01</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M02</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M03</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M04</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M05</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M06</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M07</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M08</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M09</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M10</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M11</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2340,6 +2535,45 @@
       </c>
       <c r="CR2" s="3" t="n">
         <v>-6025186534</v>
+      </c>
+      <c r="CS2" s="3" t="n">
+        <v>-26254160113</v>
+      </c>
+      <c r="CT2" s="3" t="n">
+        <v>-1780938239</v>
+      </c>
+      <c r="CU2" s="3" t="n">
+        <v>-909935447</v>
+      </c>
+      <c r="CV2" s="3" t="n">
+        <v>-3368039140</v>
+      </c>
+      <c r="CW2" s="3" t="n">
+        <v>-3129242884</v>
+      </c>
+      <c r="CX2" s="3" t="n">
+        <v>-3827815932</v>
+      </c>
+      <c r="CY2" s="3" t="n">
+        <v>1226956890</v>
+      </c>
+      <c r="CZ2" s="3" t="n">
+        <v>-1143685281</v>
+      </c>
+      <c r="DA2" s="3" t="n">
+        <v>-6353760535</v>
+      </c>
+      <c r="DB2" s="3" t="n">
+        <v>-922840649</v>
+      </c>
+      <c r="DC2" s="3" t="n">
+        <v>1715311491</v>
+      </c>
+      <c r="DD2" s="3" t="n">
+        <v>-621988193</v>
+      </c>
+      <c r="DE2" s="3" t="n">
+        <v>-7138182194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>